<commit_message>
Pondération naturelle des résultats + limites 3 étoiles du SDK
- ponderation.py remplace l'optimiseur Rust par défaut : distribution naturelle des gains,
  RTP exact 96,00 %, gros gains du bonus buy réduits juste assez pour etl40b <= 0,9
- Toutes les limites « 3 étoiles » de rgs_verification passent (base et bonus)
- run.py : --optimiseur pour revenir à l'optimiseur du SDK
- SPEC_MATHS.md : statistiques finales mises à jour

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014K11WNgkEUnnGsVcri14bC
</commit_message>
<xml_diff>
--- a/stake_math/sortie/statistiques/0_0_globe_full_statistics.xlsx
+++ b/stake_math/sortie/statistiques/0_0_globe_full_statistics.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="111">
   <si>
     <t>Win Ranges</t>
   </si>
@@ -86,94 +86,91 @@
     <t>1.007</t>
   </si>
   <si>
-    <t>1.433</t>
-  </si>
-  <si>
-    <t>35762.895</t>
-  </si>
-  <si>
-    <t>3.882</t>
-  </si>
-  <si>
-    <t>17172.792</t>
-  </si>
-  <si>
-    <t>294.724</t>
-  </si>
-  <si>
-    <t>4136.375</t>
-  </si>
-  <si>
-    <t>62.912</t>
-  </si>
-  <si>
-    <t>3235.495</t>
-  </si>
-  <si>
-    <t>64.849</t>
-  </si>
-  <si>
-    <t>1548.519</t>
-  </si>
-  <si>
-    <t>150.882</t>
-  </si>
-  <si>
-    <t>521.93</t>
-  </si>
-  <si>
-    <t>598.677</t>
-  </si>
-  <si>
-    <t>348.85</t>
-  </si>
-  <si>
-    <t>731.212</t>
-  </si>
-  <si>
-    <t>2183.821</t>
-  </si>
-  <si>
-    <t>5800.223</t>
-  </si>
-  <si>
-    <t>170122.1</t>
-  </si>
-  <si>
-    <t>3791024.014</t>
-  </si>
-  <si>
-    <t>383277.468</t>
-  </si>
-  <si>
-    <t>771042.289</t>
-  </si>
-  <si>
-    <t>154834.176</t>
-  </si>
-  <si>
-    <t>152790.601</t>
-  </si>
-  <si>
-    <t>236055.257</t>
-  </si>
-  <si>
-    <t>982520.35</t>
-  </si>
-  <si>
-    <t>1795880.082</t>
+    <t>1.417</t>
+  </si>
+  <si>
+    <t>16968.178</t>
+  </si>
+  <si>
+    <t>5.489</t>
+  </si>
+  <si>
+    <t>4363.246</t>
+  </si>
+  <si>
+    <t>12.59</t>
+  </si>
+  <si>
+    <t>638.301</t>
+  </si>
+  <si>
+    <t>35.723</t>
+  </si>
+  <si>
+    <t>405.883</t>
+  </si>
+  <si>
+    <t>295.737</t>
+  </si>
+  <si>
+    <t>665.419</t>
+  </si>
+  <si>
+    <t>1572.678</t>
+  </si>
+  <si>
+    <t>5553.222</t>
+  </si>
+  <si>
+    <t>11358.586</t>
+  </si>
+  <si>
+    <t>16509.579</t>
+  </si>
+  <si>
+    <t>3762.872</t>
+  </si>
+  <si>
+    <t>7102.958</t>
+  </si>
+  <si>
+    <t>6666.401</t>
+  </si>
+  <si>
+    <t>68151.515</t>
+  </si>
+  <si>
+    <t>19704.981</t>
+  </si>
+  <si>
+    <t>22717.172</t>
+  </si>
+  <si>
+    <t>7732.334</t>
+  </si>
+  <si>
+    <t>4259.47</t>
+  </si>
+  <si>
+    <t>12217.088</t>
+  </si>
+  <si>
+    <t>34075.758</t>
+  </si>
+  <si>
+    <t>87264.917</t>
   </si>
   <si>
     <t>NaN</t>
   </si>
   <si>
-    <t>6557234.554</t>
-  </si>
-  <si>
-    <t>14596870.76</t>
-  </si>
-  <si>
-    <t>10000002.725</t>
+    <t>305427.21</t>
+  </si>
+  <si>
+    <t>610854.42</t>
+  </si>
+  <si>
+    <t>9999999.998</t>
   </si>
   <si>
     <t>HIT RATES</t>
@@ -284,64 +281,64 @@
     <t>{'symbol': 'scatter'}</t>
   </si>
   <si>
-    <t>9.952725061834807</t>
+    <t>10.027747166612821</t>
   </si>
   <si>
     <t>4038</t>
   </si>
   <si>
-    <t>129.28470414923834</t>
-  </si>
-  <si>
-    <t>1379.575</t>
-  </si>
-  <si>
-    <t>61.454</t>
-  </si>
-  <si>
-    <t>40.488</t>
-  </si>
-  <si>
-    <t>14.153</t>
-  </si>
-  <si>
-    <t>8.0</t>
-  </si>
-  <si>
-    <t>3.996</t>
-  </si>
-  <si>
-    <t>4.499</t>
-  </si>
-  <si>
-    <t>17.679</t>
-  </si>
-  <si>
-    <t>6.099</t>
-  </si>
-  <si>
-    <t>14.611</t>
-  </si>
-  <si>
-    <t>1986.397</t>
-  </si>
-  <si>
-    <t>3155.494</t>
-  </si>
-  <si>
-    <t>3837.433</t>
-  </si>
-  <si>
-    <t>18184.034</t>
-  </si>
-  <si>
-    <t>52839.89</t>
-  </si>
-  <si>
-    <t>729478.421</t>
-  </si>
-  <si>
-    <t>169491.53</t>
+    <t>103.26357079537192</t>
+  </si>
+  <si>
+    <t>2483.577</t>
+  </si>
+  <si>
+    <t>101.629</t>
+  </si>
+  <si>
+    <t>28.606</t>
+  </si>
+  <si>
+    <t>4.208</t>
+  </si>
+  <si>
+    <t>2.588</t>
+  </si>
+  <si>
+    <t>4.684</t>
+  </si>
+  <si>
+    <t>34.644</t>
+  </si>
+  <si>
+    <t>85.756</t>
+  </si>
+  <si>
+    <t>44.714</t>
+  </si>
+  <si>
+    <t>94.234</t>
+  </si>
+  <si>
+    <t>115.961</t>
+  </si>
+  <si>
+    <t>56.524</t>
+  </si>
+  <si>
+    <t>65.728</t>
+  </si>
+  <si>
+    <t>484.543</t>
+  </si>
+  <si>
+    <t>10485.494</t>
+  </si>
+  <si>
+    <t>91134.993</t>
+  </si>
+  <si>
+    <t>91907.113</t>
   </si>
   <si>
     <t>1.0</t>
@@ -350,7 +347,7 @@
     <t>40000</t>
   </si>
   <si>
-    <t>5663.999999840501</t>
+    <t>5663.9999999996735</t>
   </si>
 </sst>
 </file>
@@ -705,7 +702,7 @@
         <v>0</v>
       </c>
       <c r="L1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:12">
@@ -713,7 +710,7 @@
         <v>3</v>
       </c>
       <c r="B2">
-        <v>1.443</v>
+        <v>1.428</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -739,10 +736,10 @@
         <v>4</v>
       </c>
       <c r="B3">
-        <v>3.895</v>
+        <v>5.516</v>
       </c>
       <c r="C3">
-        <v>0.1634885986792983</v>
+        <v>0.1040485217415406</v>
       </c>
       <c r="F3" t="s">
         <v>4</v>
@@ -765,10 +762,10 @@
         <v>5</v>
       </c>
       <c r="B4">
-        <v>327.637</v>
+        <v>12.603</v>
       </c>
       <c r="C4">
-        <v>0.004125687103350881</v>
+        <v>0.1037408691367308</v>
       </c>
       <c r="F4" t="s">
         <v>5</v>
@@ -791,10 +788,10 @@
         <v>6</v>
       </c>
       <c r="B5">
-        <v>62.618</v>
+        <v>34.001</v>
       </c>
       <c r="C5">
-        <v>0.05167028330922675</v>
+        <v>0.08392440399930619</v>
       </c>
       <c r="F5" t="s">
         <v>6</v>
@@ -817,10 +814,10 @@
         <v>7</v>
       </c>
       <c r="B6">
-        <v>63.682</v>
+        <v>171.082</v>
       </c>
       <c r="C6">
-        <v>0.1071099702685456</v>
+        <v>0.03798100187715786</v>
       </c>
       <c r="F6" t="s">
         <v>7</v>
@@ -843,10 +840,10 @@
         <v>8</v>
       </c>
       <c r="B7">
-        <v>139.831</v>
+        <v>454.026</v>
       </c>
       <c r="C7">
-        <v>0.1012566428146112</v>
+        <v>0.02962977716989274</v>
       </c>
       <c r="F7" t="s">
         <v>8</v>
@@ -869,10 +866,10 @@
         <v>9</v>
       </c>
       <c r="B8">
-        <v>281.664</v>
+        <v>3597.937</v>
       </c>
       <c r="C8">
-        <v>0.1157859651947966</v>
+        <v>0.008189708864617486</v>
       </c>
       <c r="F8" t="s">
         <v>9</v>
@@ -895,10 +892,10 @@
         <v>10</v>
       </c>
       <c r="B9">
-        <v>231.762</v>
+        <v>3049.13</v>
       </c>
       <c r="C9">
-        <v>0.3171067300152901</v>
+        <v>0.02645716456422308</v>
       </c>
       <c r="F9" t="s">
         <v>10</v>
@@ -921,10 +918,10 @@
         <v>11</v>
       </c>
       <c r="B10">
-        <v>1587.686</v>
+        <v>3458.349</v>
       </c>
       <c r="C10">
-        <v>0.07637837294147118</v>
+        <v>0.03986780927239278</v>
       </c>
       <c r="F10" t="s">
         <v>11</v>
@@ -947,19 +944,19 @@
         <v>12</v>
       </c>
       <c r="B11">
-        <v>151182.47</v>
+        <v>13007.092</v>
       </c>
       <c r="C11">
-        <v>0.001511113555760044</v>
+        <v>0.01840506887966599</v>
       </c>
       <c r="F11" t="s">
         <v>12</v>
       </c>
       <c r="G11" t="s">
+        <v>36</v>
+      </c>
+      <c r="H11" t="s">
         <v>40</v>
-      </c>
-      <c r="H11" t="s">
-        <v>41</v>
       </c>
       <c r="K11" t="s">
         <v>12</v>
@@ -973,19 +970,19 @@
         <v>13</v>
       </c>
       <c r="B12">
-        <v>256014.969</v>
+        <v>10552.068</v>
       </c>
       <c r="C12">
-        <v>0.001486603943009053</v>
+        <v>0.03660178478231444</v>
       </c>
       <c r="F12" t="s">
         <v>13</v>
       </c>
       <c r="G12" t="s">
+        <v>41</v>
+      </c>
+      <c r="H12" t="s">
         <v>42</v>
-      </c>
-      <c r="H12" t="s">
-        <v>43</v>
       </c>
       <c r="K12" t="s">
         <v>13</v>
@@ -999,19 +996,19 @@
         <v>14</v>
       </c>
       <c r="B13">
-        <v>76902.8</v>
+        <v>2746.513</v>
       </c>
       <c r="C13">
-        <v>0.009570461834816498</v>
+        <v>0.2671287960480729</v>
       </c>
       <c r="F13" t="s">
         <v>14</v>
       </c>
       <c r="G13" t="s">
+        <v>43</v>
+      </c>
+      <c r="H13" t="s">
         <v>44</v>
-      </c>
-      <c r="H13" t="s">
-        <v>45</v>
       </c>
       <c r="K13" t="s">
         <v>14</v>
@@ -1025,19 +1022,19 @@
         <v>15</v>
       </c>
       <c r="B14">
-        <v>190328.029</v>
+        <v>8992.892</v>
       </c>
       <c r="C14">
-        <v>0.007160207848634482</v>
+        <v>0.1524572349588424</v>
       </c>
       <c r="F14" t="s">
         <v>15</v>
       </c>
       <c r="G14" t="s">
+        <v>45</v>
+      </c>
+      <c r="H14" t="s">
         <v>46</v>
-      </c>
-      <c r="H14" t="s">
-        <v>47</v>
       </c>
       <c r="K14" t="s">
         <v>15</v>
@@ -1051,19 +1048,19 @@
         <v>16</v>
       </c>
       <c r="B15">
-        <v>1795880.082</v>
+        <v>87264.917</v>
       </c>
       <c r="C15">
-        <v>0.001277069975703363</v>
+        <v>0.02615631397084294</v>
       </c>
       <c r="F15" t="s">
         <v>16</v>
       </c>
       <c r="G15" t="s">
+        <v>47</v>
+      </c>
+      <c r="H15" t="s">
         <v>48</v>
-      </c>
-      <c r="H15" t="s">
-        <v>49</v>
       </c>
       <c r="K15" t="s">
         <v>16</v>
@@ -1077,19 +1074,19 @@
         <v>17</v>
       </c>
       <c r="B16">
-        <v>6557234.554</v>
+        <v>305427.21</v>
       </c>
       <c r="C16">
-        <v>0.000511610604087052</v>
+        <v>0.01101358978461481</v>
       </c>
       <c r="F16" t="s">
         <v>17</v>
       </c>
       <c r="G16" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H16" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="K16" t="s">
         <v>17</v>
@@ -1103,19 +1100,19 @@
         <v>18</v>
       </c>
       <c r="B17">
-        <v>14596870.76</v>
+        <v>610854.42</v>
       </c>
       <c r="C17">
-        <v>0.0005606818156265546</v>
+        <v>0.01339795494972198</v>
       </c>
       <c r="F17" t="s">
         <v>18</v>
       </c>
       <c r="G17" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H17" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="K17" t="s">
         <v>18</v>
@@ -1129,19 +1126,19 @@
         <v>19</v>
       </c>
       <c r="B18">
-        <v>10256413.051</v>
+        <v>10256410.255</v>
       </c>
       <c r="C18">
-        <v>0.0009750099843003219</v>
+        <v>0.0009750102501633543</v>
       </c>
       <c r="F18" t="s">
         <v>19</v>
       </c>
       <c r="G18" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H18" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="K18" t="s">
         <v>19</v>
@@ -1152,245 +1149,245 @@
     </row>
     <row r="22" spans="1:70">
       <c r="A22" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="Y22" t="s">
+        <v>81</v>
+      </c>
+      <c r="AW22" t="s">
         <v>82</v>
-      </c>
-      <c r="AW22" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="23" spans="1:70">
       <c r="B23" t="s">
+        <v>60</v>
+      </c>
+      <c r="C23" t="s">
         <v>61</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>62</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23" t="s">
         <v>63</v>
       </c>
-      <c r="E23" t="s">
+      <c r="F23" t="s">
         <v>64</v>
       </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
         <v>65</v>
       </c>
-      <c r="G23" t="s">
+      <c r="H23" t="s">
         <v>66</v>
       </c>
-      <c r="H23" t="s">
+      <c r="I23" t="s">
         <v>67</v>
       </c>
-      <c r="I23" t="s">
+      <c r="J23" t="s">
         <v>68</v>
       </c>
-      <c r="J23" t="s">
+      <c r="K23" t="s">
         <v>69</v>
       </c>
-      <c r="K23" t="s">
+      <c r="L23" t="s">
         <v>70</v>
       </c>
-      <c r="L23" t="s">
+      <c r="M23" t="s">
         <v>71</v>
       </c>
-      <c r="M23" t="s">
+      <c r="N23" t="s">
         <v>72</v>
       </c>
-      <c r="N23" t="s">
+      <c r="O23" t="s">
         <v>73</v>
       </c>
-      <c r="O23" t="s">
+      <c r="P23" t="s">
         <v>74</v>
       </c>
-      <c r="P23" t="s">
+      <c r="Q23" t="s">
         <v>75</v>
       </c>
-      <c r="Q23" t="s">
+      <c r="R23" t="s">
         <v>76</v>
       </c>
-      <c r="R23" t="s">
+      <c r="S23" t="s">
         <v>77</v>
       </c>
-      <c r="S23" t="s">
+      <c r="T23" t="s">
         <v>78</v>
       </c>
-      <c r="T23" t="s">
+      <c r="U23" t="s">
         <v>79</v>
       </c>
-      <c r="U23" t="s">
+      <c r="V23" t="s">
         <v>80</v>
       </c>
-      <c r="V23" t="s">
-        <v>81</v>
-      </c>
       <c r="Z23" t="s">
+        <v>60</v>
+      </c>
+      <c r="AA23" t="s">
         <v>61</v>
       </c>
-      <c r="AA23" t="s">
+      <c r="AB23" t="s">
         <v>62</v>
       </c>
-      <c r="AB23" t="s">
+      <c r="AC23" t="s">
         <v>63</v>
       </c>
-      <c r="AC23" t="s">
+      <c r="AD23" t="s">
         <v>64</v>
       </c>
-      <c r="AD23" t="s">
+      <c r="AE23" t="s">
         <v>65</v>
       </c>
-      <c r="AE23" t="s">
+      <c r="AF23" t="s">
         <v>66</v>
       </c>
-      <c r="AF23" t="s">
+      <c r="AG23" t="s">
         <v>67</v>
       </c>
-      <c r="AG23" t="s">
+      <c r="AH23" t="s">
         <v>68</v>
       </c>
-      <c r="AH23" t="s">
+      <c r="AI23" t="s">
         <v>69</v>
       </c>
-      <c r="AI23" t="s">
+      <c r="AJ23" t="s">
         <v>70</v>
       </c>
-      <c r="AJ23" t="s">
+      <c r="AK23" t="s">
         <v>71</v>
       </c>
-      <c r="AK23" t="s">
+      <c r="AL23" t="s">
         <v>72</v>
       </c>
-      <c r="AL23" t="s">
+      <c r="AM23" t="s">
         <v>73</v>
       </c>
-      <c r="AM23" t="s">
+      <c r="AN23" t="s">
         <v>74</v>
       </c>
-      <c r="AN23" t="s">
+      <c r="AO23" t="s">
         <v>75</v>
       </c>
-      <c r="AO23" t="s">
+      <c r="AP23" t="s">
         <v>76</v>
       </c>
-      <c r="AP23" t="s">
+      <c r="AQ23" t="s">
         <v>77</v>
       </c>
-      <c r="AQ23" t="s">
+      <c r="AR23" t="s">
         <v>78</v>
       </c>
-      <c r="AR23" t="s">
+      <c r="AS23" t="s">
         <v>79</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AT23" t="s">
         <v>80</v>
       </c>
-      <c r="AT23" t="s">
-        <v>81</v>
-      </c>
       <c r="AX23" t="s">
+        <v>60</v>
+      </c>
+      <c r="AY23" t="s">
         <v>61</v>
       </c>
-      <c r="AY23" t="s">
+      <c r="AZ23" t="s">
         <v>62</v>
       </c>
-      <c r="AZ23" t="s">
+      <c r="BA23" t="s">
         <v>63</v>
       </c>
-      <c r="BA23" t="s">
+      <c r="BB23" t="s">
         <v>64</v>
       </c>
-      <c r="BB23" t="s">
+      <c r="BC23" t="s">
         <v>65</v>
       </c>
-      <c r="BC23" t="s">
+      <c r="BD23" t="s">
         <v>66</v>
       </c>
-      <c r="BD23" t="s">
+      <c r="BE23" t="s">
         <v>67</v>
       </c>
-      <c r="BE23" t="s">
+      <c r="BF23" t="s">
         <v>68</v>
       </c>
-      <c r="BF23" t="s">
+      <c r="BG23" t="s">
         <v>69</v>
       </c>
-      <c r="BG23" t="s">
+      <c r="BH23" t="s">
         <v>70</v>
       </c>
-      <c r="BH23" t="s">
+      <c r="BI23" t="s">
         <v>71</v>
       </c>
-      <c r="BI23" t="s">
+      <c r="BJ23" t="s">
         <v>72</v>
       </c>
-      <c r="BJ23" t="s">
+      <c r="BK23" t="s">
         <v>73</v>
       </c>
-      <c r="BK23" t="s">
+      <c r="BL23" t="s">
         <v>74</v>
       </c>
-      <c r="BL23" t="s">
+      <c r="BM23" t="s">
         <v>75</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BN23" t="s">
         <v>76</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BO23" t="s">
         <v>77</v>
       </c>
-      <c r="BO23" t="s">
+      <c r="BP23" t="s">
         <v>78</v>
       </c>
-      <c r="BP23" t="s">
+      <c r="BQ23" t="s">
         <v>79</v>
       </c>
-      <c r="BQ23" t="s">
+      <c r="BR23" t="s">
         <v>80</v>
-      </c>
-      <c r="BR23" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="24" spans="1:70">
       <c r="A24" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B24">
-        <v>1207.76</v>
+        <v>1418.34</v>
       </c>
       <c r="C24">
-        <v>3838.11</v>
+        <v>3579.49</v>
       </c>
       <c r="D24">
-        <v>720.8200000000001</v>
+        <v>667.5</v>
       </c>
       <c r="E24">
-        <v>7665.74</v>
+        <v>7596.73</v>
       </c>
       <c r="F24">
-        <v>7576.3</v>
+        <v>6844.76</v>
       </c>
       <c r="G24">
-        <v>706.6799999999999</v>
+        <v>732.5599999999999</v>
       </c>
       <c r="H24">
-        <v>3711.22</v>
+        <v>3205.23</v>
       </c>
       <c r="I24">
-        <v>39254.04</v>
+        <v>68151.52</v>
       </c>
       <c r="J24">
-        <v>2411364.14</v>
+        <v>68151.52</v>
       </c>
       <c r="K24">
-        <v>80220</v>
+        <v>61311.18</v>
       </c>
       <c r="L24">
-        <v>14531.6</v>
+        <v>17099.52</v>
       </c>
       <c r="M24">
-        <v>9800.799999999999</v>
+        <v>9776.209999999999</v>
       </c>
       <c r="N24">
         <v>0</v>
@@ -1420,7 +1417,7 @@
         <v>0</v>
       </c>
       <c r="Y24" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="Z24">
         <v>26</v>
@@ -1486,28 +1483,28 @@
         <v>0</v>
       </c>
       <c r="AW24" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="AX24">
-        <v>29.6</v>
+        <v>23.3</v>
       </c>
       <c r="AY24">
-        <v>26.1</v>
+        <v>40.7</v>
       </c>
       <c r="AZ24">
-        <v>43.3</v>
+        <v>44.8</v>
       </c>
       <c r="BA24">
-        <v>22.5</v>
+        <v>29</v>
       </c>
       <c r="BB24">
-        <v>3.7</v>
+        <v>25.1</v>
       </c>
       <c r="BC24">
-        <v>39.2</v>
+        <v>46.6</v>
       </c>
       <c r="BD24">
-        <v>22.1</v>
+        <v>48.1</v>
       </c>
       <c r="BE24">
         <v>80</v>
@@ -1516,13 +1513,13 @@
         <v>100</v>
       </c>
       <c r="BG24">
-        <v>49.1</v>
+        <v>105.2</v>
       </c>
       <c r="BH24">
-        <v>29.6</v>
+        <v>20.1</v>
       </c>
       <c r="BI24">
-        <v>9</v>
+        <v>8.6</v>
       </c>
       <c r="BJ24">
         <v>0</v>
@@ -1554,43 +1551,43 @@
     </row>
     <row r="25" spans="1:70">
       <c r="A25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B25">
-        <v>412.52</v>
+        <v>409.22</v>
       </c>
       <c r="C25">
-        <v>1879.88</v>
+        <v>1840.69</v>
       </c>
       <c r="D25">
-        <v>639.21</v>
+        <v>587.79</v>
       </c>
       <c r="E25">
-        <v>2917.23</v>
+        <v>3417.43</v>
       </c>
       <c r="F25">
-        <v>5768.28</v>
+        <v>5706.72</v>
       </c>
       <c r="G25">
-        <v>715.1900000000001</v>
+        <v>714.84</v>
       </c>
       <c r="H25">
-        <v>1595.09</v>
+        <v>1590.79</v>
       </c>
       <c r="I25">
-        <v>9135.57</v>
+        <v>7596.73</v>
       </c>
       <c r="J25">
-        <v>44076.59</v>
+        <v>32275.32</v>
       </c>
       <c r="K25">
-        <v>45513.54</v>
+        <v>68151.52</v>
       </c>
       <c r="L25">
         <v>0</v>
       </c>
       <c r="M25">
-        <v>6809.4</v>
+        <v>11385.95</v>
       </c>
       <c r="N25">
         <v>0</v>
@@ -1620,7 +1617,7 @@
         <v>0</v>
       </c>
       <c r="Y25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="Z25">
         <v>97</v>
@@ -1686,34 +1683,34 @@
         <v>0</v>
       </c>
       <c r="AW25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="AX25">
-        <v>78</v>
+        <v>49.8</v>
       </c>
       <c r="AY25">
-        <v>46.4</v>
+        <v>56.6</v>
       </c>
       <c r="AZ25">
-        <v>15.5</v>
+        <v>28</v>
       </c>
       <c r="BA25">
-        <v>62.7</v>
+        <v>69.7</v>
       </c>
       <c r="BB25">
         <v>0</v>
       </c>
       <c r="BC25">
-        <v>22.6</v>
+        <v>32</v>
       </c>
       <c r="BD25">
-        <v>26.1</v>
+        <v>25.9</v>
       </c>
       <c r="BE25">
-        <v>11.1</v>
+        <v>39</v>
       </c>
       <c r="BF25">
-        <v>62.4</v>
+        <v>146.5</v>
       </c>
       <c r="BG25">
         <v>50</v>
@@ -1722,7 +1719,7 @@
         <v>0</v>
       </c>
       <c r="BI25">
-        <v>61.7</v>
+        <v>45.1</v>
       </c>
       <c r="BJ25">
         <v>0</v>
@@ -1754,46 +1751,46 @@
     </row>
     <row r="26" spans="1:70">
       <c r="A26" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B26">
-        <v>135.14</v>
+        <v>131.94</v>
       </c>
       <c r="C26">
-        <v>548.5599999999999</v>
+        <v>521.78</v>
       </c>
       <c r="D26">
-        <v>527.24</v>
+        <v>491.97</v>
       </c>
       <c r="E26">
-        <v>2542.76</v>
+        <v>2261.42</v>
       </c>
       <c r="F26">
-        <v>2959.45</v>
+        <v>2712.8</v>
       </c>
       <c r="G26">
-        <v>785.77</v>
+        <v>773.1900000000001</v>
       </c>
       <c r="H26">
-        <v>1647.62</v>
+        <v>1615.33</v>
       </c>
       <c r="I26">
-        <v>4309.34</v>
+        <v>4278.75</v>
       </c>
       <c r="J26">
-        <v>14943.66</v>
+        <v>11177.61</v>
       </c>
       <c r="K26">
-        <v>5702543.15</v>
+        <v>610854.42</v>
       </c>
       <c r="L26">
-        <v>8268.370000000001</v>
+        <v>8549.76</v>
       </c>
       <c r="M26">
-        <v>8729.82</v>
+        <v>11385.95</v>
       </c>
       <c r="N26">
-        <v>23073.13</v>
+        <v>22826.9</v>
       </c>
       <c r="O26">
         <v>0</v>
@@ -1820,7 +1817,7 @@
         <v>0</v>
       </c>
       <c r="Y26" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="Z26">
         <v>308</v>
@@ -1886,43 +1883,43 @@
         <v>0</v>
       </c>
       <c r="AW26" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="AX26">
-        <v>65.09999999999999</v>
+        <v>248.5</v>
       </c>
       <c r="AY26">
-        <v>44.2</v>
+        <v>47.4</v>
       </c>
       <c r="AZ26">
-        <v>55.8</v>
+        <v>689</v>
       </c>
       <c r="BA26">
-        <v>88.5</v>
+        <v>1026.3</v>
       </c>
       <c r="BB26">
-        <v>135.8</v>
+        <v>94.3</v>
       </c>
       <c r="BC26">
-        <v>21.8</v>
+        <v>29.1</v>
       </c>
       <c r="BD26">
-        <v>38.2</v>
+        <v>47.6</v>
       </c>
       <c r="BE26">
-        <v>4</v>
+        <v>3.8</v>
       </c>
       <c r="BF26">
-        <v>21.8</v>
+        <v>77</v>
       </c>
       <c r="BG26">
         <v>690</v>
       </c>
       <c r="BH26">
-        <v>13.1</v>
+        <v>11.3</v>
       </c>
       <c r="BI26">
-        <v>42.2</v>
+        <v>33.4</v>
       </c>
       <c r="BJ26">
         <v>0</v>
@@ -1954,49 +1951,49 @@
     </row>
     <row r="27" spans="1:70">
       <c r="A27" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B27">
-        <v>29.37</v>
+        <v>29.26</v>
       </c>
       <c r="C27">
-        <v>103.15</v>
+        <v>101.51</v>
       </c>
       <c r="D27">
-        <v>238.05</v>
+        <v>235.74</v>
       </c>
       <c r="E27">
-        <v>785.33</v>
+        <v>738.61</v>
       </c>
       <c r="F27">
-        <v>1567.7</v>
+        <v>1415.48</v>
       </c>
       <c r="G27">
-        <v>511.81</v>
+        <v>507.97</v>
       </c>
       <c r="H27">
-        <v>918.83</v>
+        <v>851.4</v>
       </c>
       <c r="I27">
-        <v>2810.89</v>
+        <v>2849.92</v>
       </c>
       <c r="J27">
-        <v>4287.56</v>
+        <v>4527.17</v>
       </c>
       <c r="K27">
-        <v>23092.36</v>
+        <v>21902.63</v>
       </c>
       <c r="L27">
         <v>0</v>
       </c>
       <c r="M27">
-        <v>4075.77</v>
+        <v>6211.88</v>
       </c>
       <c r="N27">
         <v>0</v>
       </c>
       <c r="O27">
-        <v>10103.94</v>
+        <v>9776.209999999999</v>
       </c>
       <c r="P27">
         <v>0</v>
@@ -2020,7 +2017,7 @@
         <v>0</v>
       </c>
       <c r="Y27" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="Z27">
         <v>1381</v>
@@ -2086,49 +2083,49 @@
         <v>0</v>
       </c>
       <c r="AW27" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AX27">
-        <v>101.9</v>
+        <v>61.9</v>
       </c>
       <c r="AY27">
-        <v>164.5</v>
+        <v>100.8</v>
       </c>
       <c r="AZ27">
-        <v>60.3</v>
+        <v>435.1</v>
       </c>
       <c r="BA27">
-        <v>24.9</v>
+        <v>39.4</v>
       </c>
       <c r="BB27">
-        <v>71.90000000000001</v>
+        <v>55.9</v>
       </c>
       <c r="BC27">
-        <v>149</v>
+        <v>114.6</v>
       </c>
       <c r="BD27">
-        <v>20.5</v>
+        <v>32.5</v>
       </c>
       <c r="BE27">
-        <v>23.2</v>
+        <v>26.8</v>
       </c>
       <c r="BF27">
-        <v>16</v>
+        <v>16.6</v>
       </c>
       <c r="BG27">
-        <v>59.6</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="BH27">
         <v>0</v>
       </c>
       <c r="BI27">
-        <v>50.5</v>
+        <v>31</v>
       </c>
       <c r="BJ27">
         <v>0</v>
       </c>
       <c r="BK27">
-        <v>5</v>
+        <v>5.7</v>
       </c>
       <c r="BL27">
         <v>0</v>
@@ -2154,46 +2151,46 @@
     </row>
     <row r="28" spans="1:70">
       <c r="A28" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B28">
-        <v>6.57</v>
+        <v>6.51</v>
       </c>
       <c r="C28">
-        <v>12.9</v>
+        <v>12.94</v>
       </c>
       <c r="D28">
-        <v>27.23</v>
+        <v>26.95</v>
       </c>
       <c r="E28">
-        <v>64.08</v>
+        <v>63.73</v>
       </c>
       <c r="F28">
-        <v>154.36</v>
+        <v>153.27</v>
       </c>
       <c r="G28">
-        <v>227.04</v>
+        <v>243.2</v>
       </c>
       <c r="H28">
-        <v>537.1799999999999</v>
+        <v>515.11</v>
       </c>
       <c r="I28">
-        <v>652.77</v>
+        <v>643.45</v>
       </c>
       <c r="J28">
-        <v>1650.15</v>
+        <v>1619.61</v>
       </c>
       <c r="K28">
-        <v>5931.44</v>
+        <v>5159.59</v>
       </c>
       <c r="L28">
-        <v>6040.51</v>
+        <v>6027.98</v>
       </c>
       <c r="M28">
-        <v>4222.64</v>
+        <v>5647.15</v>
       </c>
       <c r="N28">
-        <v>24402.71</v>
+        <v>32275.32</v>
       </c>
       <c r="O28">
         <v>0</v>
@@ -2202,7 +2199,7 @@
         <v>0</v>
       </c>
       <c r="Q28">
-        <v>23073.13</v>
+        <v>22826.9</v>
       </c>
       <c r="R28">
         <v>0</v>
@@ -2220,7 +2217,7 @@
         <v>0</v>
       </c>
       <c r="Y28" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="Z28">
         <v>6172</v>
@@ -2286,46 +2283,46 @@
         <v>0</v>
       </c>
       <c r="AW28" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="AX28">
-        <v>97.59999999999999</v>
+        <v>91.8</v>
       </c>
       <c r="AY28">
-        <v>120.9</v>
+        <v>117.8</v>
       </c>
       <c r="AZ28">
-        <v>95.59999999999999</v>
+        <v>101.6</v>
       </c>
       <c r="BA28">
-        <v>48.3</v>
+        <v>165.8</v>
       </c>
       <c r="BB28">
-        <v>90.3</v>
+        <v>66.5</v>
       </c>
       <c r="BC28">
-        <v>109.9</v>
+        <v>36.2</v>
       </c>
       <c r="BD28">
-        <v>180.7</v>
+        <v>155.7</v>
       </c>
       <c r="BE28">
-        <v>12.9</v>
+        <v>19</v>
       </c>
       <c r="BF28">
-        <v>22.2</v>
+        <v>36</v>
       </c>
       <c r="BG28">
-        <v>55.1</v>
+        <v>88</v>
       </c>
       <c r="BH28">
-        <v>32.7</v>
+        <v>53.6</v>
       </c>
       <c r="BI28">
-        <v>39.1</v>
+        <v>35.4</v>
       </c>
       <c r="BJ28">
-        <v>74.59999999999999</v>
+        <v>100.1</v>
       </c>
       <c r="BK28">
         <v>0</v>
@@ -2354,52 +2351,52 @@
     </row>
     <row r="29" spans="1:70">
       <c r="A29" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B29">
-        <v>5.11</v>
+        <v>5.13</v>
       </c>
       <c r="C29">
         <v>9.359999999999999</v>
       </c>
       <c r="D29">
-        <v>16.93</v>
+        <v>16.94</v>
       </c>
       <c r="E29">
-        <v>32.25</v>
+        <v>32.42</v>
       </c>
       <c r="F29">
-        <v>69.98</v>
+        <v>71.45</v>
       </c>
       <c r="G29">
-        <v>132.23</v>
+        <v>130.63</v>
       </c>
       <c r="H29">
-        <v>229.51</v>
+        <v>228.68</v>
       </c>
       <c r="I29">
-        <v>587.04</v>
+        <v>593.03</v>
       </c>
       <c r="J29">
-        <v>1061.37</v>
+        <v>1002.13</v>
       </c>
       <c r="K29">
-        <v>1744.65</v>
+        <v>1788.39</v>
       </c>
       <c r="L29">
-        <v>2806.4</v>
+        <v>2618.69</v>
       </c>
       <c r="M29">
-        <v>8916.15</v>
+        <v>9776.209999999999</v>
       </c>
       <c r="N29">
-        <v>3149.37</v>
+        <v>4271.02</v>
       </c>
       <c r="O29">
-        <v>10707.07</v>
+        <v>11385.95</v>
       </c>
       <c r="P29">
-        <v>35805.15</v>
+        <v>68151.52</v>
       </c>
       <c r="Q29">
         <v>0</v>
@@ -2420,7 +2417,7 @@
         <v>0</v>
       </c>
       <c r="Y29" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="Z29">
         <v>7848</v>
@@ -2486,49 +2483,49 @@
         <v>0</v>
       </c>
       <c r="AW29" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="AX29">
-        <v>113.2</v>
+        <v>89.3</v>
       </c>
       <c r="AY29">
-        <v>115.7</v>
+        <v>107.1</v>
       </c>
       <c r="AZ29">
-        <v>86.2</v>
+        <v>77</v>
       </c>
       <c r="BA29">
-        <v>118.8</v>
+        <v>150.8</v>
       </c>
       <c r="BB29">
-        <v>190</v>
+        <v>108.9</v>
       </c>
       <c r="BC29">
-        <v>132.6</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="BD29">
-        <v>127.3</v>
+        <v>157.2</v>
       </c>
       <c r="BE29">
-        <v>49.6</v>
+        <v>113</v>
       </c>
       <c r="BF29">
-        <v>19.7</v>
+        <v>33</v>
       </c>
       <c r="BG29">
+        <v>32.2</v>
+      </c>
+      <c r="BH29">
+        <v>3464.4</v>
+      </c>
+      <c r="BI29">
+        <v>11.5</v>
+      </c>
+      <c r="BJ29">
+        <v>35.1</v>
+      </c>
+      <c r="BK29">
         <v>26.7</v>
-      </c>
-      <c r="BH29">
-        <v>116.5</v>
-      </c>
-      <c r="BI29">
-        <v>18.2</v>
-      </c>
-      <c r="BJ29">
-        <v>46.9</v>
-      </c>
-      <c r="BK29">
-        <v>32.3</v>
       </c>
       <c r="BL29">
         <v>70</v>
@@ -2554,58 +2551,58 @@
     </row>
     <row r="30" spans="1:70">
       <c r="A30" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B30">
-        <v>4.2</v>
+        <v>4.21</v>
       </c>
       <c r="C30">
-        <v>7.15</v>
+        <v>7.21</v>
       </c>
       <c r="D30">
-        <v>12.36</v>
+        <v>12.38</v>
       </c>
       <c r="E30">
-        <v>21.75</v>
+        <v>22.09</v>
       </c>
       <c r="F30">
-        <v>43.46</v>
+        <v>44.33</v>
       </c>
       <c r="G30">
-        <v>80.43000000000001</v>
+        <v>78.75</v>
       </c>
       <c r="H30">
-        <v>145.65</v>
+        <v>154.27</v>
       </c>
       <c r="I30">
-        <v>305.07</v>
+        <v>310.06</v>
       </c>
       <c r="J30">
-        <v>782.27</v>
+        <v>755.79</v>
       </c>
       <c r="K30">
-        <v>879.58</v>
+        <v>988.02</v>
       </c>
       <c r="L30">
-        <v>2896.51</v>
+        <v>2709.69</v>
       </c>
       <c r="M30">
-        <v>1464.75</v>
+        <v>3970.27</v>
       </c>
       <c r="N30">
-        <v>8902.23</v>
+        <v>9622.209999999999</v>
       </c>
       <c r="O30">
-        <v>14031.27</v>
+        <v>17099.52</v>
       </c>
       <c r="P30">
-        <v>7880.21</v>
+        <v>8549.76</v>
       </c>
       <c r="Q30">
-        <v>45513.54</v>
+        <v>68151.52</v>
       </c>
       <c r="R30">
-        <v>23073.13</v>
+        <v>22826.9</v>
       </c>
       <c r="S30">
         <v>0</v>
@@ -2620,7 +2617,7 @@
         <v>0</v>
       </c>
       <c r="Y30" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="Z30">
         <v>9519</v>
@@ -2686,52 +2683,52 @@
         <v>0</v>
       </c>
       <c r="AW30" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="AX30">
-        <v>108.7</v>
+        <v>88.8</v>
       </c>
       <c r="AY30">
-        <v>107.3</v>
+        <v>109</v>
       </c>
       <c r="AZ30">
-        <v>119.8</v>
+        <v>126.8</v>
       </c>
       <c r="BA30">
-        <v>92.59999999999999</v>
+        <v>96</v>
       </c>
       <c r="BB30">
-        <v>187</v>
+        <v>109.9</v>
       </c>
       <c r="BC30">
-        <v>87.7</v>
+        <v>61.5</v>
       </c>
       <c r="BD30">
-        <v>75.8</v>
+        <v>39.6</v>
       </c>
       <c r="BE30">
-        <v>106</v>
+        <v>107.8</v>
       </c>
       <c r="BF30">
-        <v>28</v>
+        <v>39.4</v>
       </c>
       <c r="BG30">
-        <v>87.09999999999999</v>
+        <v>34.6</v>
       </c>
       <c r="BH30">
-        <v>25.3</v>
+        <v>41.7</v>
       </c>
       <c r="BI30">
-        <v>505.7</v>
+        <v>97.8</v>
       </c>
       <c r="BJ30">
-        <v>19.2</v>
+        <v>22.2</v>
       </c>
       <c r="BK30">
-        <v>27.4</v>
+        <v>17.6</v>
       </c>
       <c r="BL30">
-        <v>19.3</v>
+        <v>13.8</v>
       </c>
       <c r="BM30">
         <v>50</v>
@@ -2754,32 +2751,32 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="B36" t="s">
+        <v>84</v>
+      </c>
+      <c r="C36" t="s">
         <v>85</v>
       </c>
-      <c r="C36" t="s">
+      <c r="D36" t="s">
         <v>86</v>
-      </c>
-      <c r="D36" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" t="s">
+        <v>87</v>
+      </c>
+      <c r="B37" t="s">
         <v>88</v>
       </c>
-      <c r="B37" t="s">
+      <c r="C37" t="s">
         <v>89</v>
       </c>
-      <c r="C37" t="s">
+      <c r="D37" t="s">
         <v>90</v>
-      </c>
-      <c r="D37" t="s">
-        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -2809,7 +2806,7 @@
         <v>0</v>
       </c>
       <c r="K1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:11">
@@ -2817,7 +2814,7 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -2826,7 +2823,7 @@
         <v>3</v>
       </c>
       <c r="G2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="J2" t="s">
         <v>3</v>
@@ -2840,16 +2837,16 @@
         <v>4</v>
       </c>
       <c r="B3">
-        <v>64.798</v>
+        <v>119.332</v>
       </c>
       <c r="C3">
-        <v>0.0001712726535061315</v>
+        <v>9.029634298164544E-05</v>
       </c>
       <c r="F3" t="s">
         <v>4</v>
       </c>
       <c r="G3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J3" t="s">
         <v>4</v>
@@ -2863,16 +2860,16 @@
         <v>5</v>
       </c>
       <c r="B4">
-        <v>40.9</v>
+        <v>31.067</v>
       </c>
       <c r="C4">
-        <v>0.0005993534739676811</v>
+        <v>0.0008153375544101675</v>
       </c>
       <c r="F4" t="s">
         <v>5</v>
       </c>
       <c r="G4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="J4" t="s">
         <v>5</v>
@@ -2886,16 +2883,16 @@
         <v>6</v>
       </c>
       <c r="B5">
-        <v>14.549</v>
+        <v>4.39</v>
       </c>
       <c r="C5">
-        <v>0.004021706709759511</v>
+        <v>0.01389760522475812</v>
       </c>
       <c r="F5" t="s">
         <v>6</v>
       </c>
       <c r="G5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="J5" t="s">
         <v>6</v>
@@ -2909,16 +2906,16 @@
         <v>7</v>
       </c>
       <c r="B6">
-        <v>8.272</v>
+        <v>2.564</v>
       </c>
       <c r="C6">
-        <v>0.01536035447865712</v>
+        <v>0.04790064397482078</v>
       </c>
       <c r="F6" t="s">
         <v>7</v>
       </c>
       <c r="G6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J6" t="s">
         <v>7</v>
@@ -2932,16 +2929,16 @@
         <v>8</v>
       </c>
       <c r="B7">
-        <v>4.017</v>
+        <v>4.488</v>
       </c>
       <c r="C7">
-        <v>0.06286645593138958</v>
+        <v>0.04987782012386114</v>
       </c>
       <c r="F7" t="s">
         <v>8</v>
       </c>
       <c r="G7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J7" t="s">
         <v>8</v>
@@ -2955,16 +2952,16 @@
         <v>9</v>
       </c>
       <c r="B8">
-        <v>4.34</v>
+        <v>33.056</v>
       </c>
       <c r="C8">
-        <v>0.1023334831254502</v>
+        <v>0.01399924811065666</v>
       </c>
       <c r="F8" t="s">
         <v>9</v>
       </c>
       <c r="G8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J8" t="s">
         <v>9</v>
@@ -2978,16 +2975,16 @@
         <v>10</v>
       </c>
       <c r="B9">
-        <v>17.568</v>
+        <v>85.018</v>
       </c>
       <c r="C9">
-        <v>0.07133374253786609</v>
+        <v>0.0150516889372899</v>
       </c>
       <c r="F9" t="s">
         <v>10</v>
       </c>
       <c r="G9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J9" t="s">
         <v>10</v>
@@ -3001,16 +2998,16 @@
         <v>11</v>
       </c>
       <c r="B10">
-        <v>6.098</v>
+        <v>44.512</v>
       </c>
       <c r="C10">
-        <v>0.4308670204231783</v>
+        <v>0.05629920102043136</v>
       </c>
       <c r="F10" t="s">
         <v>11</v>
       </c>
       <c r="G10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J10" t="s">
         <v>11</v>
@@ -3024,16 +3021,16 @@
         <v>12</v>
       </c>
       <c r="B11">
-        <v>14.475</v>
+        <v>94.236</v>
       </c>
       <c r="C11">
-        <v>0.2549723937534055</v>
+        <v>0.04291881084771184</v>
       </c>
       <c r="F11" t="s">
         <v>12</v>
       </c>
       <c r="G11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="J11" t="s">
         <v>12</v>
@@ -3047,16 +3044,16 @@
         <v>13</v>
       </c>
       <c r="B12">
-        <v>1936.586</v>
+        <v>115.262</v>
       </c>
       <c r="C12">
-        <v>0.002978758943555864</v>
+        <v>0.05693742198485256</v>
       </c>
       <c r="F12" t="s">
         <v>13</v>
       </c>
       <c r="G12" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="J12" t="s">
         <v>13</v>
@@ -3070,16 +3067,16 @@
         <v>14</v>
       </c>
       <c r="B13">
-        <v>3155.494</v>
+        <v>56.524</v>
       </c>
       <c r="C13">
-        <v>0.003964669210794382</v>
+        <v>0.2225566501436065</v>
       </c>
       <c r="F13" t="s">
         <v>14</v>
       </c>
       <c r="G13" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="J13" t="s">
         <v>14</v>
@@ -3093,16 +3090,16 @@
         <v>15</v>
       </c>
       <c r="B14">
-        <v>3837.433</v>
+        <v>65.72799999999999</v>
       </c>
       <c r="C14">
-        <v>0.006032376249319595</v>
+        <v>0.3540162012131984</v>
       </c>
       <c r="F14" t="s">
         <v>15</v>
       </c>
       <c r="G14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="J14" t="s">
         <v>15</v>
@@ -3116,16 +3113,16 @@
         <v>16</v>
       </c>
       <c r="B15">
-        <v>18184.034</v>
+        <v>484.543</v>
       </c>
       <c r="C15">
-        <v>0.002196364048206984</v>
+        <v>0.07678595519986857</v>
       </c>
       <c r="F15" t="s">
         <v>16</v>
       </c>
       <c r="G15" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="J15" t="s">
         <v>16</v>
@@ -3139,16 +3136,16 @@
         <v>17</v>
       </c>
       <c r="B16">
-        <v>52839.89</v>
+        <v>10485.494</v>
       </c>
       <c r="C16">
-        <v>0.001138098598716005</v>
+        <v>0.005724719335969995</v>
       </c>
       <c r="F16" t="s">
         <v>17</v>
       </c>
       <c r="G16" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="J16" t="s">
         <v>17</v>
@@ -3162,16 +3159,16 @@
         <v>18</v>
       </c>
       <c r="B17">
-        <v>729478.421</v>
+        <v>91134.993</v>
       </c>
       <c r="C17">
-        <v>0.0001639498626439739</v>
+        <v>0.001284238848229411</v>
       </c>
       <c r="F17" t="s">
         <v>18</v>
       </c>
       <c r="G17" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="J17" t="s">
         <v>18</v>
@@ -3185,16 +3182,16 @@
         <v>19</v>
       </c>
       <c r="B18">
-        <v>179999.091</v>
+        <v>94919.364</v>
       </c>
       <c r="C18">
-        <v>0.000941630938632813</v>
+        <v>0.001785643580119753</v>
       </c>
       <c r="F18" t="s">
         <v>19</v>
       </c>
       <c r="G18" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="J18" t="s">
         <v>19</v>
@@ -3205,251 +3202,251 @@
     </row>
     <row r="22" spans="1:70">
       <c r="A22" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="Y22" t="s">
+        <v>81</v>
+      </c>
+      <c r="AW22" t="s">
         <v>82</v>
-      </c>
-      <c r="AW22" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="23" spans="1:70">
       <c r="B23" t="s">
+        <v>60</v>
+      </c>
+      <c r="C23" t="s">
         <v>61</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>62</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23" t="s">
         <v>63</v>
       </c>
-      <c r="E23" t="s">
+      <c r="F23" t="s">
         <v>64</v>
       </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
         <v>65</v>
       </c>
-      <c r="G23" t="s">
+      <c r="H23" t="s">
         <v>66</v>
       </c>
-      <c r="H23" t="s">
+      <c r="I23" t="s">
         <v>67</v>
       </c>
-      <c r="I23" t="s">
+      <c r="J23" t="s">
         <v>68</v>
       </c>
-      <c r="J23" t="s">
+      <c r="K23" t="s">
         <v>69</v>
       </c>
-      <c r="K23" t="s">
+      <c r="L23" t="s">
         <v>70</v>
       </c>
-      <c r="L23" t="s">
+      <c r="M23" t="s">
         <v>71</v>
       </c>
-      <c r="M23" t="s">
+      <c r="N23" t="s">
         <v>72</v>
       </c>
-      <c r="N23" t="s">
+      <c r="O23" t="s">
         <v>73</v>
       </c>
-      <c r="O23" t="s">
+      <c r="P23" t="s">
         <v>74</v>
       </c>
-      <c r="P23" t="s">
+      <c r="Q23" t="s">
         <v>75</v>
       </c>
-      <c r="Q23" t="s">
+      <c r="R23" t="s">
         <v>76</v>
       </c>
-      <c r="R23" t="s">
+      <c r="S23" t="s">
         <v>77</v>
       </c>
-      <c r="S23" t="s">
+      <c r="T23" t="s">
         <v>78</v>
       </c>
-      <c r="T23" t="s">
+      <c r="U23" t="s">
         <v>79</v>
       </c>
-      <c r="U23" t="s">
+      <c r="V23" t="s">
         <v>80</v>
       </c>
-      <c r="V23" t="s">
-        <v>81</v>
-      </c>
       <c r="Z23" t="s">
+        <v>60</v>
+      </c>
+      <c r="AA23" t="s">
         <v>61</v>
       </c>
-      <c r="AA23" t="s">
+      <c r="AB23" t="s">
         <v>62</v>
       </c>
-      <c r="AB23" t="s">
+      <c r="AC23" t="s">
         <v>63</v>
       </c>
-      <c r="AC23" t="s">
+      <c r="AD23" t="s">
         <v>64</v>
       </c>
-      <c r="AD23" t="s">
+      <c r="AE23" t="s">
         <v>65</v>
       </c>
-      <c r="AE23" t="s">
+      <c r="AF23" t="s">
         <v>66</v>
       </c>
-      <c r="AF23" t="s">
+      <c r="AG23" t="s">
         <v>67</v>
       </c>
-      <c r="AG23" t="s">
+      <c r="AH23" t="s">
         <v>68</v>
       </c>
-      <c r="AH23" t="s">
+      <c r="AI23" t="s">
         <v>69</v>
       </c>
-      <c r="AI23" t="s">
+      <c r="AJ23" t="s">
         <v>70</v>
       </c>
-      <c r="AJ23" t="s">
+      <c r="AK23" t="s">
         <v>71</v>
       </c>
-      <c r="AK23" t="s">
+      <c r="AL23" t="s">
         <v>72</v>
       </c>
-      <c r="AL23" t="s">
+      <c r="AM23" t="s">
         <v>73</v>
       </c>
-      <c r="AM23" t="s">
+      <c r="AN23" t="s">
         <v>74</v>
       </c>
-      <c r="AN23" t="s">
+      <c r="AO23" t="s">
         <v>75</v>
       </c>
-      <c r="AO23" t="s">
+      <c r="AP23" t="s">
         <v>76</v>
       </c>
-      <c r="AP23" t="s">
+      <c r="AQ23" t="s">
         <v>77</v>
       </c>
-      <c r="AQ23" t="s">
+      <c r="AR23" t="s">
         <v>78</v>
       </c>
-      <c r="AR23" t="s">
+      <c r="AS23" t="s">
         <v>79</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AT23" t="s">
         <v>80</v>
       </c>
-      <c r="AT23" t="s">
-        <v>81</v>
-      </c>
       <c r="AX23" t="s">
+        <v>60</v>
+      </c>
+      <c r="AY23" t="s">
         <v>61</v>
       </c>
-      <c r="AY23" t="s">
+      <c r="AZ23" t="s">
         <v>62</v>
       </c>
-      <c r="AZ23" t="s">
+      <c r="BA23" t="s">
         <v>63</v>
       </c>
-      <c r="BA23" t="s">
+      <c r="BB23" t="s">
         <v>64</v>
       </c>
-      <c r="BB23" t="s">
+      <c r="BC23" t="s">
         <v>65</v>
       </c>
-      <c r="BC23" t="s">
+      <c r="BD23" t="s">
         <v>66</v>
       </c>
-      <c r="BD23" t="s">
+      <c r="BE23" t="s">
         <v>67</v>
       </c>
-      <c r="BE23" t="s">
+      <c r="BF23" t="s">
         <v>68</v>
       </c>
-      <c r="BF23" t="s">
+      <c r="BG23" t="s">
         <v>69</v>
       </c>
-      <c r="BG23" t="s">
+      <c r="BH23" t="s">
         <v>70</v>
       </c>
-      <c r="BH23" t="s">
+      <c r="BI23" t="s">
         <v>71</v>
       </c>
-      <c r="BI23" t="s">
+      <c r="BJ23" t="s">
         <v>72</v>
       </c>
-      <c r="BJ23" t="s">
+      <c r="BK23" t="s">
         <v>73</v>
       </c>
-      <c r="BK23" t="s">
+      <c r="BL23" t="s">
         <v>74</v>
       </c>
-      <c r="BL23" t="s">
+      <c r="BM23" t="s">
         <v>75</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BN23" t="s">
         <v>76</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BO23" t="s">
         <v>77</v>
       </c>
-      <c r="BO23" t="s">
+      <c r="BP23" t="s">
         <v>78</v>
       </c>
-      <c r="BP23" t="s">
+      <c r="BQ23" t="s">
         <v>79</v>
       </c>
-      <c r="BQ23" t="s">
+      <c r="BR23" t="s">
         <v>80</v>
-      </c>
-      <c r="BR23" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="24" spans="1:70">
       <c r="A24" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B24">
-        <v>171.35</v>
+        <v>239.78</v>
       </c>
       <c r="C24">
-        <v>925.84</v>
+        <v>746.71</v>
       </c>
       <c r="D24">
-        <v>96.33</v>
+        <v>95.27</v>
       </c>
       <c r="E24">
-        <v>519.12</v>
+        <v>825.35</v>
       </c>
       <c r="F24">
-        <v>822.38</v>
+        <v>628.92</v>
       </c>
       <c r="G24">
-        <v>72.23</v>
+        <v>89.91</v>
       </c>
       <c r="H24">
-        <v>437.99</v>
+        <v>392.21</v>
       </c>
       <c r="I24">
-        <v>4061.37</v>
+        <v>1796.94</v>
       </c>
       <c r="J24">
-        <v>2069.87</v>
+        <v>1564.25</v>
       </c>
       <c r="K24">
-        <v>2665.45</v>
+        <v>2333.68</v>
       </c>
       <c r="L24">
-        <v>5849.74</v>
+        <v>3026.72</v>
       </c>
       <c r="M24">
-        <v>4365.22</v>
+        <v>2627.29</v>
       </c>
       <c r="N24">
-        <v>13763.19</v>
+        <v>9928.75</v>
       </c>
       <c r="O24">
-        <v>142647.73</v>
+        <v>39707.82</v>
       </c>
       <c r="P24">
         <v>0</v>
@@ -3473,7 +3470,7 @@
         <v>0</v>
       </c>
       <c r="Y24" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="Z24">
         <v>167</v>
@@ -3539,46 +3536,46 @@
         <v>0</v>
       </c>
       <c r="AW24" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="AX24">
-        <v>6855.5</v>
+        <v>4241.4</v>
       </c>
       <c r="AY24">
-        <v>4459.4</v>
+        <v>4445.2</v>
       </c>
       <c r="AZ24">
-        <v>5446.7</v>
+        <v>5011.5</v>
       </c>
       <c r="BA24">
-        <v>3422.7</v>
+        <v>1641.7</v>
       </c>
       <c r="BB24">
-        <v>6025.2</v>
+        <v>3138.2</v>
       </c>
       <c r="BC24">
-        <v>8030.5</v>
+        <v>4438.3</v>
       </c>
       <c r="BD24">
-        <v>3547.9</v>
+        <v>3371.6</v>
       </c>
       <c r="BE24">
-        <v>1058.4</v>
+        <v>5571.1</v>
       </c>
       <c r="BF24">
-        <v>1800.6</v>
+        <v>17401.1</v>
       </c>
       <c r="BG24">
-        <v>7410.5</v>
+        <v>1744.9</v>
       </c>
       <c r="BH24">
-        <v>1418.7</v>
+        <v>10658.9</v>
       </c>
       <c r="BI24">
-        <v>1510.9</v>
+        <v>8955.5</v>
       </c>
       <c r="BJ24">
-        <v>790.3</v>
+        <v>645.2</v>
       </c>
       <c r="BK24">
         <v>830</v>
@@ -3607,52 +3604,52 @@
     </row>
     <row r="25" spans="1:70">
       <c r="A25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B25">
-        <v>64.72</v>
+        <v>70.92</v>
       </c>
       <c r="C25">
-        <v>320.6</v>
+        <v>286.98</v>
       </c>
       <c r="D25">
-        <v>81.84</v>
+        <v>81.33</v>
       </c>
       <c r="E25">
-        <v>587.34</v>
+        <v>420.33</v>
       </c>
       <c r="F25">
-        <v>639.4299999999999</v>
+        <v>513.09</v>
       </c>
       <c r="G25">
-        <v>70.06</v>
+        <v>81.87</v>
       </c>
       <c r="H25">
-        <v>233.36</v>
+        <v>251.05</v>
       </c>
       <c r="I25">
-        <v>975.21</v>
+        <v>1092.95</v>
       </c>
       <c r="J25">
-        <v>1283.11</v>
+        <v>1587.33</v>
       </c>
       <c r="K25">
-        <v>742.6900000000001</v>
+        <v>2300.79</v>
       </c>
       <c r="L25">
-        <v>6753.23</v>
+        <v>3309.43</v>
       </c>
       <c r="M25">
-        <v>2520.97</v>
+        <v>2335.84</v>
       </c>
       <c r="N25">
-        <v>4456.38</v>
+        <v>4962.76</v>
       </c>
       <c r="O25">
-        <v>80051.67</v>
+        <v>19860.79</v>
       </c>
       <c r="P25">
-        <v>11287.5</v>
+        <v>19614.78</v>
       </c>
       <c r="Q25">
         <v>0</v>
@@ -3673,7 +3670,7 @@
         <v>0</v>
       </c>
       <c r="Y25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="Z25">
         <v>562</v>
@@ -3739,52 +3736,52 @@
         <v>0</v>
       </c>
       <c r="AW25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="AX25">
-        <v>5087.1</v>
+        <v>4404.7</v>
       </c>
       <c r="AY25">
-        <v>2728.3</v>
+        <v>3607.7</v>
       </c>
       <c r="AZ25">
-        <v>5487.6</v>
+        <v>5413.6</v>
       </c>
       <c r="BA25">
-        <v>2954.2</v>
+        <v>6330.8</v>
       </c>
       <c r="BB25">
-        <v>3907.1</v>
+        <v>6178.2</v>
       </c>
       <c r="BC25">
-        <v>7333</v>
+        <v>7037.9</v>
       </c>
       <c r="BD25">
-        <v>5829.9</v>
+        <v>8278.200000000001</v>
       </c>
       <c r="BE25">
-        <v>2185.9</v>
+        <v>10925.9</v>
       </c>
       <c r="BF25">
-        <v>13311</v>
+        <v>1467.3</v>
       </c>
       <c r="BG25">
-        <v>16883.1</v>
+        <v>16629.5</v>
       </c>
       <c r="BH25">
-        <v>720.7</v>
+        <v>691.8</v>
       </c>
       <c r="BI25">
-        <v>1475.8</v>
+        <v>792</v>
       </c>
       <c r="BJ25">
-        <v>1305</v>
+        <v>979.1</v>
       </c>
       <c r="BK25">
-        <v>475.7</v>
+        <v>475</v>
       </c>
       <c r="BL25">
-        <v>22699.8</v>
+        <v>13319.4</v>
       </c>
       <c r="BM25">
         <v>0</v>
@@ -3807,52 +3804,52 @@
     </row>
     <row r="26" spans="1:70">
       <c r="A26" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B26">
-        <v>17.38</v>
+        <v>19.53</v>
       </c>
       <c r="C26">
-        <v>85.13</v>
+        <v>87</v>
       </c>
       <c r="D26">
-        <v>71.89</v>
+        <v>65.14</v>
       </c>
       <c r="E26">
-        <v>169.7</v>
+        <v>208.27</v>
       </c>
       <c r="F26">
-        <v>337.34</v>
+        <v>327.5</v>
       </c>
       <c r="G26">
-        <v>57.93</v>
+        <v>70.18000000000001</v>
       </c>
       <c r="H26">
-        <v>131.09</v>
+        <v>163.7</v>
       </c>
       <c r="I26">
-        <v>443.61</v>
+        <v>494.76</v>
       </c>
       <c r="J26">
-        <v>1290.42</v>
+        <v>1082.51</v>
       </c>
       <c r="K26">
-        <v>3096.02</v>
+        <v>1367.3</v>
       </c>
       <c r="L26">
-        <v>1166.67</v>
+        <v>1303.52</v>
       </c>
       <c r="M26">
-        <v>1655.78</v>
+        <v>2202.49</v>
       </c>
       <c r="N26">
-        <v>7151.8</v>
+        <v>3309.01</v>
       </c>
       <c r="O26">
-        <v>10283.59</v>
+        <v>19844.42</v>
       </c>
       <c r="P26">
-        <v>164398.06</v>
+        <v>39720.23</v>
       </c>
       <c r="Q26">
         <v>0</v>
@@ -3873,7 +3870,7 @@
         <v>0</v>
       </c>
       <c r="Y26" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="Z26">
         <v>2045</v>
@@ -3939,49 +3936,49 @@
         <v>0</v>
       </c>
       <c r="AW26" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="AX26">
-        <v>6854.9</v>
+        <v>5681.5</v>
       </c>
       <c r="AY26">
-        <v>6246.5</v>
+        <v>4158.2</v>
       </c>
       <c r="AZ26">
-        <v>4714.4</v>
+        <v>3438.9</v>
       </c>
       <c r="BA26">
-        <v>6021.6</v>
+        <v>3666.6</v>
       </c>
       <c r="BB26">
-        <v>9538.5</v>
+        <v>2940.8</v>
       </c>
       <c r="BC26">
-        <v>6960</v>
+        <v>5826.4</v>
       </c>
       <c r="BD26">
-        <v>8859.700000000001</v>
+        <v>7088.3</v>
       </c>
       <c r="BE26">
-        <v>3747.1</v>
+        <v>4214</v>
       </c>
       <c r="BF26">
-        <v>8058.9</v>
+        <v>19109.1</v>
       </c>
       <c r="BG26">
-        <v>1089</v>
+        <v>2304.6</v>
       </c>
       <c r="BH26">
-        <v>6006.5</v>
+        <v>17518.4</v>
       </c>
       <c r="BI26">
-        <v>5763.3</v>
+        <v>2470.5</v>
       </c>
       <c r="BJ26">
-        <v>991.1</v>
+        <v>821.8</v>
       </c>
       <c r="BK26">
-        <v>1929.6</v>
+        <v>1320.5</v>
       </c>
       <c r="BL26">
         <v>510</v>
@@ -4007,52 +4004,52 @@
     </row>
     <row r="27" spans="1:70">
       <c r="A27" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B27">
         <v>5.07</v>
       </c>
       <c r="C27">
-        <v>17.98</v>
+        <v>16.48</v>
       </c>
       <c r="D27">
-        <v>32.15</v>
+        <v>30.35</v>
       </c>
       <c r="E27">
-        <v>92.83</v>
+        <v>91.48</v>
       </c>
       <c r="F27">
-        <v>175.15</v>
+        <v>188.3</v>
       </c>
       <c r="G27">
-        <v>50.56</v>
+        <v>61.03</v>
       </c>
       <c r="H27">
-        <v>127.88</v>
+        <v>132.24</v>
       </c>
       <c r="I27">
-        <v>356.28</v>
+        <v>325.64</v>
       </c>
       <c r="J27">
-        <v>442.71</v>
+        <v>489.21</v>
       </c>
       <c r="K27">
-        <v>890.4400000000001</v>
+        <v>873.36</v>
       </c>
       <c r="L27">
-        <v>1200.4</v>
+        <v>1405.51</v>
       </c>
       <c r="M27">
-        <v>2181.12</v>
+        <v>1272.15</v>
       </c>
       <c r="N27">
-        <v>1627.31</v>
+        <v>2446.98</v>
       </c>
       <c r="O27">
-        <v>3505.1</v>
+        <v>5574.1</v>
       </c>
       <c r="P27">
-        <v>29634.42</v>
+        <v>13239.08</v>
       </c>
       <c r="Q27">
         <v>0</v>
@@ -4073,7 +4070,7 @@
         <v>0</v>
       </c>
       <c r="Y27" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="Z27">
         <v>7901</v>
@@ -4139,52 +4136,52 @@
         <v>0</v>
       </c>
       <c r="AW27" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="AX27">
-        <v>5436.3</v>
+        <v>5275.1</v>
       </c>
       <c r="AY27">
-        <v>5136.1</v>
+        <v>6106.1</v>
       </c>
       <c r="AZ27">
-        <v>5593.6</v>
+        <v>5074.8</v>
       </c>
       <c r="BA27">
-        <v>4809.8</v>
+        <v>5613.3</v>
       </c>
       <c r="BB27">
-        <v>6079.5</v>
+        <v>4992.6</v>
       </c>
       <c r="BC27">
-        <v>6884.5</v>
+        <v>6318.7</v>
       </c>
       <c r="BD27">
-        <v>8088.2</v>
+        <v>5393.3</v>
       </c>
       <c r="BE27">
-        <v>3658.7</v>
+        <v>9169.299999999999</v>
       </c>
       <c r="BF27">
-        <v>3646.1</v>
+        <v>2995</v>
       </c>
       <c r="BG27">
-        <v>7446.5</v>
+        <v>10039.7</v>
       </c>
       <c r="BH27">
-        <v>14041.4</v>
+        <v>10374.5</v>
       </c>
       <c r="BI27">
-        <v>1438.2</v>
+        <v>8532.4</v>
       </c>
       <c r="BJ27">
-        <v>8532.700000000001</v>
+        <v>16409</v>
       </c>
       <c r="BK27">
-        <v>7932</v>
+        <v>19523.3</v>
       </c>
       <c r="BL27">
-        <v>539.4</v>
+        <v>586.8</v>
       </c>
       <c r="BM27">
         <v>0</v>
@@ -4207,55 +4204,55 @@
     </row>
     <row r="28" spans="1:70">
       <c r="A28" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B28">
-        <v>1.39</v>
+        <v>1.4</v>
       </c>
       <c r="C28">
         <v>2.45</v>
       </c>
       <c r="D28">
-        <v>4.81</v>
+        <v>4.71</v>
       </c>
       <c r="E28">
-        <v>11.04</v>
+        <v>10.66</v>
       </c>
       <c r="F28">
-        <v>23.04</v>
+        <v>23.84</v>
       </c>
       <c r="G28">
-        <v>30.23</v>
+        <v>33.95</v>
       </c>
       <c r="H28">
-        <v>56.06</v>
+        <v>63.47</v>
       </c>
       <c r="I28">
-        <v>89.33</v>
+        <v>104.62</v>
       </c>
       <c r="J28">
-        <v>190.83</v>
+        <v>162.68</v>
       </c>
       <c r="K28">
-        <v>326.46</v>
+        <v>337.73</v>
       </c>
       <c r="L28">
-        <v>769.6799999999999</v>
+        <v>598.51</v>
       </c>
       <c r="M28">
-        <v>691.75</v>
+        <v>636.54</v>
       </c>
       <c r="N28">
-        <v>1433.43</v>
+        <v>1098.89</v>
       </c>
       <c r="O28">
-        <v>2518.79</v>
+        <v>2821.29</v>
       </c>
       <c r="P28">
-        <v>3215.43</v>
+        <v>3970.06</v>
       </c>
       <c r="Q28">
-        <v>26452.39</v>
+        <v>7617.39</v>
       </c>
       <c r="R28">
         <v>0</v>
@@ -4273,7 +4270,7 @@
         <v>0</v>
       </c>
       <c r="Y28" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="Z28">
         <v>28495</v>
@@ -4339,55 +4336,55 @@
         <v>0</v>
       </c>
       <c r="AW28" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="AX28">
-        <v>5711.5</v>
+        <v>5585.3</v>
       </c>
       <c r="AY28">
-        <v>5621.5</v>
+        <v>5733.1</v>
       </c>
       <c r="AZ28">
-        <v>5546.8</v>
+        <v>5548.1</v>
       </c>
       <c r="BA28">
-        <v>5926.7</v>
+        <v>5256.1</v>
       </c>
       <c r="BB28">
-        <v>5914.3</v>
+        <v>5540.4</v>
       </c>
       <c r="BC28">
-        <v>5903.1</v>
+        <v>5779.7</v>
       </c>
       <c r="BD28">
-        <v>7506.6</v>
+        <v>5126.5</v>
       </c>
       <c r="BE28">
-        <v>8146.1</v>
+        <v>7627.6</v>
       </c>
       <c r="BF28">
-        <v>5979.1</v>
+        <v>5654.8</v>
       </c>
       <c r="BG28">
-        <v>4482.4</v>
+        <v>6037.6</v>
       </c>
       <c r="BH28">
-        <v>6132.4</v>
+        <v>6377.7</v>
       </c>
       <c r="BI28">
-        <v>6760.5</v>
+        <v>7357.5</v>
       </c>
       <c r="BJ28">
-        <v>6603.3</v>
+        <v>4828</v>
       </c>
       <c r="BK28">
-        <v>1834.2</v>
+        <v>6432.3</v>
       </c>
       <c r="BL28">
-        <v>3607.9</v>
+        <v>1018.4</v>
       </c>
       <c r="BM28">
-        <v>4594.9</v>
+        <v>46873.4</v>
       </c>
       <c r="BN28">
         <v>0</v>
@@ -4407,58 +4404,58 @@
     </row>
     <row r="29" spans="1:70">
       <c r="A29" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B29">
-        <v>1.18</v>
+        <v>1.2</v>
       </c>
       <c r="C29">
-        <v>1.81</v>
+        <v>1.82</v>
       </c>
       <c r="D29">
         <v>3.07</v>
       </c>
       <c r="E29">
-        <v>5.9</v>
+        <v>5.92</v>
       </c>
       <c r="F29">
-        <v>10.9</v>
+        <v>11.76</v>
       </c>
       <c r="G29">
-        <v>21.02</v>
+        <v>21.21</v>
       </c>
       <c r="H29">
-        <v>34.95</v>
+        <v>37.67</v>
       </c>
       <c r="I29">
-        <v>60.22</v>
+        <v>66.58</v>
       </c>
       <c r="J29">
-        <v>93.75</v>
+        <v>127.31</v>
       </c>
       <c r="K29">
-        <v>174.84</v>
+        <v>225.66</v>
       </c>
       <c r="L29">
-        <v>477.36</v>
+        <v>420.02</v>
       </c>
       <c r="M29">
-        <v>515</v>
+        <v>541.9299999999999</v>
       </c>
       <c r="N29">
-        <v>1373.41</v>
+        <v>877.74</v>
       </c>
       <c r="O29">
-        <v>1683.32</v>
+        <v>2205.08</v>
       </c>
       <c r="P29">
-        <v>3158.92</v>
+        <v>3970.1</v>
       </c>
       <c r="Q29">
-        <v>21724.83</v>
+        <v>7634.09</v>
       </c>
       <c r="R29">
-        <v>66779662.85</v>
+        <v>66610169.49</v>
       </c>
       <c r="S29">
         <v>0</v>
@@ -4473,7 +4470,7 @@
         <v>0</v>
       </c>
       <c r="Y29" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="Z29">
         <v>33256</v>
@@ -4539,55 +4536,55 @@
         <v>0</v>
       </c>
       <c r="AW29" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="AX29">
-        <v>5686.2</v>
+        <v>5578.7</v>
       </c>
       <c r="AY29">
-        <v>5768.5</v>
+        <v>5462.7</v>
       </c>
       <c r="AZ29">
-        <v>5594.8</v>
+        <v>5482.8</v>
       </c>
       <c r="BA29">
-        <v>5510.1</v>
+        <v>5433.3</v>
       </c>
       <c r="BB29">
-        <v>6428.2</v>
+        <v>5090.8</v>
       </c>
       <c r="BC29">
-        <v>6386.1</v>
+        <v>5375.2</v>
       </c>
       <c r="BD29">
-        <v>7191.7</v>
+        <v>4884.9</v>
       </c>
       <c r="BE29">
-        <v>4897.9</v>
+        <v>6675.3</v>
       </c>
       <c r="BF29">
-        <v>8249</v>
+        <v>6611.3</v>
       </c>
       <c r="BG29">
-        <v>7203.4</v>
+        <v>6762.6</v>
       </c>
       <c r="BH29">
-        <v>11270.2</v>
+        <v>6049.3</v>
       </c>
       <c r="BI29">
-        <v>4740.8</v>
+        <v>4715.8</v>
       </c>
       <c r="BJ29">
-        <v>3778.7</v>
+        <v>6533.2</v>
       </c>
       <c r="BK29">
-        <v>2786.6</v>
+        <v>1252.2</v>
       </c>
       <c r="BL29">
-        <v>1829.8</v>
+        <v>1005.3</v>
       </c>
       <c r="BM29">
-        <v>2354.1</v>
+        <v>44284.5</v>
       </c>
       <c r="BN29">
         <v>1000000</v>
@@ -4607,58 +4604,58 @@
     </row>
     <row r="30" spans="1:70">
       <c r="A30" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B30">
-        <v>1.08</v>
+        <v>1.09</v>
       </c>
       <c r="C30">
-        <v>1.49</v>
+        <v>1.48</v>
       </c>
       <c r="D30">
-        <v>2.25</v>
+        <v>2.27</v>
       </c>
       <c r="E30">
-        <v>3.85</v>
+        <v>3.92</v>
       </c>
       <c r="F30">
-        <v>7.3</v>
+        <v>7.2</v>
       </c>
       <c r="G30">
-        <v>12.71</v>
+        <v>12.93</v>
       </c>
       <c r="H30">
-        <v>23.65</v>
+        <v>24.75</v>
       </c>
       <c r="I30">
-        <v>44.04</v>
+        <v>43.15</v>
       </c>
       <c r="J30">
-        <v>70.09</v>
+        <v>79.47</v>
       </c>
       <c r="K30">
-        <v>152.55</v>
+        <v>156.27</v>
       </c>
       <c r="L30">
-        <v>260.59</v>
+        <v>266.98</v>
       </c>
       <c r="M30">
-        <v>317.56</v>
+        <v>469.77</v>
       </c>
       <c r="N30">
-        <v>892.86</v>
+        <v>896.83</v>
       </c>
       <c r="O30">
-        <v>2489.66</v>
+        <v>1588.15</v>
       </c>
       <c r="P30">
-        <v>8087.43</v>
+        <v>3610.6</v>
       </c>
       <c r="Q30">
-        <v>6420.36</v>
+        <v>9925.5</v>
       </c>
       <c r="R30">
-        <v>119975.65</v>
+        <v>39722.16</v>
       </c>
       <c r="S30">
         <v>0</v>
@@ -4673,7 +4670,7 @@
         <v>0</v>
       </c>
       <c r="Y30" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="Z30">
         <v>36744</v>
@@ -4739,55 +4736,55 @@
         <v>0</v>
       </c>
       <c r="AW30" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="AX30">
-        <v>5567.9</v>
+        <v>5579.1</v>
       </c>
       <c r="AY30">
-        <v>5739.6</v>
+        <v>5690.5</v>
       </c>
       <c r="AZ30">
-        <v>5747.9</v>
+        <v>5777.2</v>
       </c>
       <c r="BA30">
-        <v>6099.4</v>
+        <v>5530.8</v>
       </c>
       <c r="BB30">
-        <v>5686.1</v>
+        <v>5564.9</v>
       </c>
       <c r="BC30">
-        <v>6321.2</v>
+        <v>5747</v>
       </c>
       <c r="BD30">
-        <v>5614.4</v>
+        <v>5774.7</v>
       </c>
       <c r="BE30">
-        <v>4138.9</v>
+        <v>4476.3</v>
       </c>
       <c r="BF30">
-        <v>7608.1</v>
+        <v>6190.1</v>
       </c>
       <c r="BG30">
-        <v>6455.9</v>
+        <v>5134.1</v>
       </c>
       <c r="BH30">
-        <v>4215.9</v>
+        <v>6212.8</v>
       </c>
       <c r="BI30">
-        <v>10705</v>
+        <v>7574.7</v>
       </c>
       <c r="BJ30">
-        <v>5847</v>
+        <v>7505.1</v>
       </c>
       <c r="BK30">
-        <v>1259.4</v>
+        <v>935.6</v>
       </c>
       <c r="BL30">
-        <v>897</v>
+        <v>604.7</v>
       </c>
       <c r="BM30">
-        <v>1790</v>
+        <v>980.5</v>
       </c>
       <c r="BN30">
         <v>460</v>
@@ -4807,32 +4804,32 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="B36" t="s">
+        <v>84</v>
+      </c>
+      <c r="C36" t="s">
         <v>85</v>
       </c>
-      <c r="C36" t="s">
+      <c r="D36" t="s">
         <v>86</v>
-      </c>
-      <c r="D36" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B37" t="s">
+        <v>108</v>
+      </c>
+      <c r="C37" t="s">
         <v>109</v>
       </c>
-      <c r="C37" t="s">
+      <c r="D37" t="s">
         <v>110</v>
-      </c>
-      <c r="D37" t="s">
-        <v>111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>